<commit_message>
Changed done at 4:39 AM
</commit_message>
<xml_diff>
--- a/outputs/ExamSchedule.xlsx
+++ b/outputs/ExamSchedule.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="40">
   <si>
     <t>Date</t>
   </si>
@@ -81,6 +81,9 @@
     <t>R101, R102</t>
   </si>
   <si>
+    <t>TBA, TBA, TBA, TBA</t>
+  </si>
+  <si>
     <t>CS101</t>
   </si>
   <si>
@@ -94,6 +97,9 @@
   </si>
   <si>
     <t>H301</t>
+  </si>
+  <si>
+    <t>TBA, TBA</t>
   </si>
   <si>
     <t>CS102</t>
@@ -667,7 +673,7 @@
         <v>21</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -678,19 +684,19 @@
         <v>18</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -701,19 +707,19 @@
         <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -724,19 +730,19 @@
         <v>18</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -747,19 +753,19 @@
         <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -770,19 +776,19 @@
         <v>18</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -793,19 +799,19 @@
         <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -831,16 +837,16 @@
         <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -854,7 +860,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>21</v>
@@ -862,50 +868,50 @@
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>21</v>
@@ -913,19 +919,19 @@
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>